<commit_message>
docs(ci): align all project documents with GitHub Actions
</commit_message>
<xml_diff>
--- a/docs/OEP-19_Initial_RTM.xlsx
+++ b/docs/OEP-19_Initial_RTM.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R40ebdc4b5bde4a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability" sheetId="2" r:id="R357be960d40c476e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planned Tests" sheetId="3" r:id="R9a65025842924821"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="4" r:id="R2a6bffb0c5f64ca9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59e04ff357ee4fef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability" sheetId="2" r:id="R819e174b95864e94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planned Tests" sheetId="3" r:id="R2885a4a55da14488"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="4" r:id="R4724156fc257423a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -575,7 +575,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7a64ce94b914b4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb95ba477a5754ca1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2903,7 +2903,7 @@
         <x:v>PROC-01</x:v>
       </x:c>
       <x:c r="C48" s="10" t="str">
-        <x:v>Jira stories, keyed Git branches/commits/PRs, teammate reviews, Jenkins CI/CD, Docker and
+        <x:v>Jira stories, keyed Git branches/commits/PRs, teammate reviews, GitHub Actions, Docker and
 static analysis. Each member implements and explains a complete functionality.</x:v>
       </x:c>
       <x:c r="D48" s="10" t="str">
@@ -3017,7 +3017,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd0ce1f326ab48ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76bd7b1ec30b4751"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8536,7 +8536,7 @@
         <x:v>ST</x:v>
       </x:c>
       <x:c r="D191" s="3" t="str">
-        <x:v>Review Jira, Git contribution, PR, Jenkins, Docker and
+        <x:v>Review Jira, Git contribution, PR, GitHub Actions, Docker and
 analysis evidence</x:v>
       </x:c>
       <x:c r="E191" s="3" t="str">
@@ -8605,7 +8605,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99650aa69b3644f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfae8c832cb64f67"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8863,7 +8863,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d5cd3a9d65e48a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R768eb902b3954068"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>